<commit_message>
data de entrada lista para ambos casos de bateria
</commit_message>
<xml_diff>
--- a/data/Escenarios_DCH_septiembre/Bateria_482/Costo_fijo/Swap_fixed_3estaciones_160kW/elmo_data.xlsx
+++ b/data/Escenarios_DCH_septiembre/Bateria_482/Costo_fijo/Swap_fixed_3estaciones_160kW/elmo_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECNO-MASTER\Desktop\Elmo_infrastructure_sizing_NP-\data\Escenarios_DCH_septiembre\Bateria_353\Costo_fijo\Swap_fixed_3estaciones_160kW\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECNO-MASTER\Desktop\Elmo_infrastructure_sizing_NP-\data\Escenarios_DCH_septiembre\Bateria_482\Costo_fijo\Swap_fixed_3estaciones_160kW\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6261EE9-CD98-4335-80CC-99278EFF72E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CDC3AF8-A7DF-4A12-A74C-E9841913896C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4185" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LHD" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1089" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1049" uniqueCount="391">
   <si>
     <t>id</t>
   </si>
@@ -219,15 +219,6 @@
     <t>distance_to_d_node_return</t>
   </si>
   <si>
-    <t>0.2</t>
-  </si>
-  <si>
-    <t>0.95</t>
-  </si>
-  <si>
-    <t>swap_time</t>
-  </si>
-  <si>
     <t>LH518B_2</t>
   </si>
   <si>
@@ -1161,9 +1152,6 @@
     <t>USD</t>
   </si>
   <si>
-    <t>h</t>
-  </si>
-  <si>
     <t>station_1</t>
   </si>
   <si>
@@ -1189,9 +1177,6 @@
   </si>
   <si>
     <t>battery_cost</t>
-  </si>
-  <si>
-    <t>charge_time</t>
   </si>
   <si>
     <t>Battery_swap</t>
@@ -1586,7 +1571,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1795,6 +1780,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2101,7 +2087,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:AE17"/>
+  <dimension ref="A1:AC17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.42578125" style="23" bestFit="1" customWidth="1"/>
@@ -2129,9 +2115,10 @@
     <col min="26" max="26" width="13.5703125" style="24" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="11.28515625" style="24" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="19.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:29" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
@@ -2219,14 +2206,8 @@
       <c r="AC1" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" t="s">
-        <v>62</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="2" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:29" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="30" t="s">
         <v>3</v>
       </c>
@@ -2314,14 +2295,8 @@
       <c r="AC2" t="s">
         <v>37</v>
       </c>
-      <c r="AD2" t="s">
-        <v>374</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="3" spans="1:31" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:29" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="31">
         <v>1</v>
       </c>
@@ -2329,16 +2304,16 @@
         <v>40</v>
       </c>
       <c r="C3" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="D3" s="29" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="E3" s="21" t="s">
         <v>52</v>
       </c>
       <c r="F3" s="21" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G3" s="9">
         <v>18</v>
@@ -2353,13 +2328,13 @@
         <v>20</v>
       </c>
       <c r="K3" s="9">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="L3" s="9">
         <v>540</v>
       </c>
       <c r="M3" s="22">
-        <v>6.26</v>
+        <v>8.73</v>
       </c>
       <c r="N3" s="35">
         <v>-1</v>
@@ -2374,7 +2349,7 @@
         <v>-1</v>
       </c>
       <c r="R3" s="22">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="S3" s="26">
         <v>0.92</v>
@@ -2386,54 +2361,48 @@
         <v>0.47</v>
       </c>
       <c r="V3" s="34">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="W3" s="34">
         <v>4</v>
       </c>
-      <c r="X3" s="24">
-        <v>360</v>
-      </c>
-      <c r="Y3" s="24">
+      <c r="X3" s="72">
+        <v>320</v>
+      </c>
+      <c r="Y3" s="72">
         <v>4</v>
       </c>
-      <c r="Z3" s="24">
-        <v>353</v>
-      </c>
-      <c r="AA3" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>61</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>61</v>
-      </c>
-      <c r="AD3">
-        <v>8.3000000000000004E-2</v>
-      </c>
-      <c r="AE3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:31" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Z3" s="72">
+        <v>482</v>
+      </c>
+      <c r="AA3" s="72">
+        <v>0.2</v>
+      </c>
+      <c r="AB3" s="34">
+        <v>0.95</v>
+      </c>
+      <c r="AC3" s="34">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="31">
         <v>2</v>
       </c>
       <c r="B4" s="38" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C4" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="D4" s="29" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="E4" s="21" t="s">
         <v>52</v>
       </c>
       <c r="F4" s="21" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G4" s="9">
         <v>18</v>
@@ -2448,13 +2417,13 @@
         <v>20</v>
       </c>
       <c r="K4" s="9">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="L4" s="9">
         <v>540</v>
       </c>
       <c r="M4" s="22">
-        <v>6.26</v>
+        <v>8.73</v>
       </c>
       <c r="N4" s="35">
         <v>-1</v>
@@ -2469,7 +2438,7 @@
         <v>-1</v>
       </c>
       <c r="R4" s="22">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="S4" s="26">
         <v>0.92</v>
@@ -2481,54 +2450,48 @@
         <v>0.47</v>
       </c>
       <c r="V4" s="34">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="W4" s="34">
         <v>4</v>
       </c>
-      <c r="X4" s="24">
-        <v>360</v>
-      </c>
-      <c r="Y4" s="24">
+      <c r="X4" s="72">
+        <v>320</v>
+      </c>
+      <c r="Y4" s="72">
         <v>4</v>
       </c>
-      <c r="Z4" s="24">
-        <v>353</v>
-      </c>
-      <c r="AA4" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB4" t="s">
-        <v>61</v>
-      </c>
-      <c r="AC4" t="s">
-        <v>61</v>
-      </c>
-      <c r="AD4">
-        <v>8.3000000000000004E-2</v>
-      </c>
-      <c r="AE4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:31" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Z4" s="72">
+        <v>482</v>
+      </c>
+      <c r="AA4" s="72">
+        <v>0.2</v>
+      </c>
+      <c r="AB4" s="34">
+        <v>0.95</v>
+      </c>
+      <c r="AC4" s="34">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="31">
         <v>3</v>
       </c>
       <c r="B5" s="38" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="D5" s="29" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="E5" s="21" t="s">
         <v>52</v>
       </c>
       <c r="F5" s="21" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G5" s="9">
         <v>18</v>
@@ -2543,13 +2506,13 @@
         <v>20</v>
       </c>
       <c r="K5" s="9">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="L5" s="9">
         <v>540</v>
       </c>
       <c r="M5" s="22">
-        <v>6.26</v>
+        <v>8.73</v>
       </c>
       <c r="N5" s="35">
         <v>-1</v>
@@ -2564,7 +2527,7 @@
         <v>-1</v>
       </c>
       <c r="R5" s="22">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="S5" s="26">
         <v>0.92</v>
@@ -2576,54 +2539,48 @@
         <v>0.47</v>
       </c>
       <c r="V5" s="34">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="W5" s="34">
         <v>4</v>
       </c>
-      <c r="X5" s="24">
-        <v>360</v>
-      </c>
-      <c r="Y5" s="24">
+      <c r="X5" s="72">
+        <v>320</v>
+      </c>
+      <c r="Y5" s="72">
         <v>4</v>
       </c>
-      <c r="Z5" s="24">
-        <v>353</v>
-      </c>
-      <c r="AA5" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB5" t="s">
-        <v>61</v>
-      </c>
-      <c r="AC5" t="s">
-        <v>61</v>
-      </c>
-      <c r="AD5">
-        <v>8.3000000000000004E-2</v>
-      </c>
-      <c r="AE5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:31" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Z5" s="72">
+        <v>482</v>
+      </c>
+      <c r="AA5" s="72">
+        <v>0.2</v>
+      </c>
+      <c r="AB5" s="34">
+        <v>0.95</v>
+      </c>
+      <c r="AC5" s="34">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="31">
         <v>4</v>
       </c>
       <c r="B6" s="38" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C6" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="D6" s="29" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="E6" s="21" t="s">
         <v>52</v>
       </c>
       <c r="F6" s="21" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G6" s="9">
         <v>18</v>
@@ -2638,13 +2595,13 @@
         <v>20</v>
       </c>
       <c r="K6" s="9">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="L6" s="9">
         <v>540</v>
       </c>
       <c r="M6" s="22">
-        <v>6.26</v>
+        <v>8.73</v>
       </c>
       <c r="N6" s="35">
         <v>-1</v>
@@ -2659,7 +2616,7 @@
         <v>-1</v>
       </c>
       <c r="R6" s="22">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="S6" s="26">
         <v>0.92</v>
@@ -2671,55 +2628,48 @@
         <v>0.47</v>
       </c>
       <c r="V6" s="34">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="W6" s="34">
         <v>4</v>
       </c>
-      <c r="X6" s="24">
-        <v>360</v>
-      </c>
-      <c r="Y6" s="24">
+      <c r="X6" s="72">
+        <v>320</v>
+      </c>
+      <c r="Y6" s="72">
         <v>4</v>
       </c>
-      <c r="Z6" s="24">
-        <v>353</v>
-      </c>
-      <c r="AA6" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB6" t="s">
-        <v>61</v>
-      </c>
-      <c r="AC6" t="s">
-        <v>61</v>
-      </c>
-      <c r="AD6">
-        <v>8.3000000000000004E-2</v>
-      </c>
-      <c r="AE6">
-        <f>AE3</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:31" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Z6" s="72">
+        <v>482</v>
+      </c>
+      <c r="AA6" s="72">
+        <v>0.2</v>
+      </c>
+      <c r="AB6" s="34">
+        <v>0.95</v>
+      </c>
+      <c r="AC6" s="34">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:29" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="31">
         <v>5</v>
       </c>
       <c r="B7" s="38" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="C7" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="D7" s="29" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="E7" s="21" t="s">
         <v>52</v>
       </c>
       <c r="F7" s="21" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G7" s="9">
         <v>18</v>
@@ -2734,13 +2684,13 @@
         <v>20</v>
       </c>
       <c r="K7" s="9">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="L7" s="9">
         <v>540</v>
       </c>
       <c r="M7" s="22">
-        <v>6.26</v>
+        <v>8.73</v>
       </c>
       <c r="N7" s="35">
         <v>-1</v>
@@ -2755,7 +2705,7 @@
         <v>-1</v>
       </c>
       <c r="R7" s="22">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="S7" s="26">
         <v>0.92</v>
@@ -2767,55 +2717,48 @@
         <v>0.47</v>
       </c>
       <c r="V7" s="34">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="W7" s="34">
         <v>4</v>
       </c>
-      <c r="X7" s="24">
-        <v>360</v>
-      </c>
-      <c r="Y7" s="24">
+      <c r="X7" s="72">
+        <v>320</v>
+      </c>
+      <c r="Y7" s="72">
         <v>4</v>
       </c>
-      <c r="Z7" s="24">
-        <v>353</v>
-      </c>
-      <c r="AA7" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB7" t="s">
-        <v>61</v>
-      </c>
-      <c r="AC7" t="s">
-        <v>61</v>
-      </c>
-      <c r="AD7">
-        <v>8.3000000000000004E-2</v>
-      </c>
-      <c r="AE7">
-        <f t="shared" ref="AE7:AE14" si="0">AE4</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:31" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Z7" s="72">
+        <v>482</v>
+      </c>
+      <c r="AA7" s="72">
+        <v>0.2</v>
+      </c>
+      <c r="AB7" s="34">
+        <v>0.95</v>
+      </c>
+      <c r="AC7" s="34">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="8" spans="1:29" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="31">
         <v>6</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="C8" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="D8" s="29" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="E8" s="21" t="s">
         <v>52</v>
       </c>
       <c r="F8" s="21" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G8" s="9">
         <v>18</v>
@@ -2830,13 +2773,13 @@
         <v>20</v>
       </c>
       <c r="K8" s="9">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="L8" s="9">
         <v>540</v>
       </c>
       <c r="M8" s="22">
-        <v>6.26</v>
+        <v>8.73</v>
       </c>
       <c r="N8" s="35">
         <v>-1</v>
@@ -2851,7 +2794,7 @@
         <v>-1</v>
       </c>
       <c r="R8" s="22">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="S8" s="26">
         <v>0.92</v>
@@ -2863,55 +2806,48 @@
         <v>0.47</v>
       </c>
       <c r="V8" s="34">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="W8" s="34">
         <v>4</v>
       </c>
-      <c r="X8" s="24">
-        <v>360</v>
-      </c>
-      <c r="Y8" s="24">
+      <c r="X8" s="72">
+        <v>320</v>
+      </c>
+      <c r="Y8" s="72">
         <v>4</v>
       </c>
-      <c r="Z8" s="24">
-        <v>353</v>
-      </c>
-      <c r="AA8" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB8" t="s">
-        <v>61</v>
-      </c>
-      <c r="AC8" t="s">
-        <v>61</v>
-      </c>
-      <c r="AD8">
-        <v>8.3000000000000004E-2</v>
-      </c>
-      <c r="AE8">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:31" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Z8" s="72">
+        <v>482</v>
+      </c>
+      <c r="AA8" s="72">
+        <v>0.2</v>
+      </c>
+      <c r="AB8" s="34">
+        <v>0.95</v>
+      </c>
+      <c r="AC8" s="34">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="9" spans="1:29" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="31">
         <v>7</v>
       </c>
       <c r="B9" s="38" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="C9" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="D9" s="29" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="E9" s="21" t="s">
         <v>52</v>
       </c>
       <c r="F9" s="21" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G9" s="9">
         <v>18</v>
@@ -2926,13 +2862,13 @@
         <v>20</v>
       </c>
       <c r="K9" s="9">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="L9" s="9">
         <v>540</v>
       </c>
       <c r="M9" s="22">
-        <v>6.26</v>
+        <v>8.73</v>
       </c>
       <c r="N9" s="35">
         <v>-1</v>
@@ -2947,7 +2883,7 @@
         <v>-1</v>
       </c>
       <c r="R9" s="22">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="S9" s="26">
         <v>0.92</v>
@@ -2959,55 +2895,48 @@
         <v>0.47</v>
       </c>
       <c r="V9" s="34">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="W9" s="34">
         <v>4</v>
       </c>
-      <c r="X9" s="24">
-        <v>360</v>
-      </c>
-      <c r="Y9" s="24">
+      <c r="X9" s="72">
+        <v>320</v>
+      </c>
+      <c r="Y9" s="72">
         <v>4</v>
       </c>
-      <c r="Z9" s="24">
-        <v>353</v>
-      </c>
-      <c r="AA9" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB9" t="s">
-        <v>61</v>
-      </c>
-      <c r="AC9" t="s">
-        <v>61</v>
-      </c>
-      <c r="AD9">
-        <v>8.3000000000000004E-2</v>
-      </c>
-      <c r="AE9">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:31" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Z9" s="72">
+        <v>482</v>
+      </c>
+      <c r="AA9" s="72">
+        <v>0.2</v>
+      </c>
+      <c r="AB9" s="34">
+        <v>0.95</v>
+      </c>
+      <c r="AC9" s="34">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="10" spans="1:29" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="31">
         <v>8</v>
       </c>
       <c r="B10" s="38" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="C10" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="D10" s="29" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="E10" s="21" t="s">
         <v>52</v>
       </c>
       <c r="F10" s="21" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G10" s="9">
         <v>18</v>
@@ -3022,13 +2951,13 @@
         <v>20</v>
       </c>
       <c r="K10" s="9">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="L10" s="9">
         <v>540</v>
       </c>
       <c r="M10" s="22">
-        <v>6.26</v>
+        <v>8.73</v>
       </c>
       <c r="N10" s="35">
         <v>-1</v>
@@ -3043,7 +2972,7 @@
         <v>-1</v>
       </c>
       <c r="R10" s="22">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="S10" s="26">
         <v>0.92</v>
@@ -3055,55 +2984,48 @@
         <v>0.47</v>
       </c>
       <c r="V10" s="34">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="W10" s="34">
         <v>4</v>
       </c>
-      <c r="X10" s="24">
-        <v>360</v>
-      </c>
-      <c r="Y10" s="24">
+      <c r="X10" s="72">
+        <v>320</v>
+      </c>
+      <c r="Y10" s="72">
         <v>4</v>
       </c>
-      <c r="Z10" s="24">
-        <v>353</v>
-      </c>
-      <c r="AA10" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB10" t="s">
-        <v>61</v>
-      </c>
-      <c r="AC10" t="s">
-        <v>61</v>
-      </c>
-      <c r="AD10">
-        <v>8.3000000000000004E-2</v>
-      </c>
-      <c r="AE10">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:31" s="34" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Z10" s="72">
+        <v>482</v>
+      </c>
+      <c r="AA10" s="72">
+        <v>0.2</v>
+      </c>
+      <c r="AB10" s="34">
+        <v>0.95</v>
+      </c>
+      <c r="AC10" s="34">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="11" spans="1:29" s="34" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="31">
         <v>9</v>
       </c>
       <c r="B11" s="38" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="C11" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="D11" s="29" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="E11" s="21" t="s">
         <v>52</v>
       </c>
       <c r="F11" s="21" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G11" s="9">
         <v>18</v>
@@ -3118,13 +3040,13 @@
         <v>20</v>
       </c>
       <c r="K11" s="9">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="L11" s="9">
         <v>540</v>
       </c>
       <c r="M11" s="22">
-        <v>6.26</v>
+        <v>8.73</v>
       </c>
       <c r="N11" s="35">
         <v>-1</v>
@@ -3139,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="R11" s="22">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="S11" s="26">
         <v>0.92</v>
@@ -3151,55 +3073,48 @@
         <v>0.47</v>
       </c>
       <c r="V11" s="34">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="W11" s="34">
         <v>4</v>
       </c>
-      <c r="X11" s="24">
-        <v>360</v>
-      </c>
-      <c r="Y11" s="24">
+      <c r="X11" s="72">
+        <v>320</v>
+      </c>
+      <c r="Y11" s="72">
         <v>4</v>
       </c>
-      <c r="Z11" s="24">
-        <v>353</v>
-      </c>
-      <c r="AA11" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB11" t="s">
-        <v>61</v>
-      </c>
-      <c r="AC11" t="s">
-        <v>61</v>
-      </c>
-      <c r="AD11">
-        <v>8.3000000000000004E-2</v>
-      </c>
-      <c r="AE11">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:31" s="34" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Z11" s="72">
+        <v>482</v>
+      </c>
+      <c r="AA11" s="72">
+        <v>0.2</v>
+      </c>
+      <c r="AB11" s="34">
+        <v>0.95</v>
+      </c>
+      <c r="AC11" s="34">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="12" spans="1:29" s="34" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="31">
         <v>10</v>
       </c>
       <c r="B12" s="38" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="C12" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="D12" s="29" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="E12" s="21" t="s">
         <v>52</v>
       </c>
       <c r="F12" s="21" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G12" s="9">
         <v>18</v>
@@ -3214,13 +3129,13 @@
         <v>20</v>
       </c>
       <c r="K12" s="9">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="L12" s="9">
         <v>540</v>
       </c>
       <c r="M12" s="22">
-        <v>6.26</v>
+        <v>8.73</v>
       </c>
       <c r="N12" s="35">
         <v>-1</v>
@@ -3235,7 +3150,7 @@
         <v>-1</v>
       </c>
       <c r="R12" s="22">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="S12" s="26">
         <v>0.92</v>
@@ -3247,55 +3162,48 @@
         <v>0.47</v>
       </c>
       <c r="V12" s="34">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="W12" s="34">
         <v>4</v>
       </c>
-      <c r="X12" s="24">
-        <v>360</v>
-      </c>
-      <c r="Y12" s="24">
+      <c r="X12" s="72">
+        <v>320</v>
+      </c>
+      <c r="Y12" s="72">
         <v>4</v>
       </c>
-      <c r="Z12" s="24">
-        <v>353</v>
-      </c>
-      <c r="AA12" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB12" t="s">
-        <v>61</v>
-      </c>
-      <c r="AC12" t="s">
-        <v>61</v>
-      </c>
-      <c r="AD12">
-        <v>8.3000000000000004E-2</v>
-      </c>
-      <c r="AE12">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:31" s="34" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Z12" s="72">
+        <v>482</v>
+      </c>
+      <c r="AA12" s="72">
+        <v>0.2</v>
+      </c>
+      <c r="AB12" s="34">
+        <v>0.95</v>
+      </c>
+      <c r="AC12" s="34">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="13" spans="1:29" s="34" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="31">
         <v>11</v>
       </c>
       <c r="B13" s="38" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="C13" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="D13" s="29" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="E13" s="21" t="s">
         <v>52</v>
       </c>
       <c r="F13" s="21" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G13" s="9">
         <v>18</v>
@@ -3310,13 +3218,13 @@
         <v>20</v>
       </c>
       <c r="K13" s="9">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="L13" s="9">
         <v>540</v>
       </c>
       <c r="M13" s="22">
-        <v>6.26</v>
+        <v>8.73</v>
       </c>
       <c r="N13" s="35">
         <v>-1</v>
@@ -3331,7 +3239,7 @@
         <v>-1</v>
       </c>
       <c r="R13" s="22">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="S13" s="26">
         <v>0.92</v>
@@ -3343,55 +3251,48 @@
         <v>0.47</v>
       </c>
       <c r="V13" s="34">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="W13" s="34">
         <v>4</v>
       </c>
-      <c r="X13" s="24">
-        <v>360</v>
-      </c>
-      <c r="Y13" s="24">
+      <c r="X13" s="72">
+        <v>320</v>
+      </c>
+      <c r="Y13" s="72">
         <v>4</v>
       </c>
-      <c r="Z13" s="24">
-        <v>353</v>
-      </c>
-      <c r="AA13" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB13" t="s">
-        <v>61</v>
-      </c>
-      <c r="AC13" t="s">
-        <v>61</v>
-      </c>
-      <c r="AD13">
-        <v>8.3000000000000004E-2</v>
-      </c>
-      <c r="AE13">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:31" s="34" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Z13" s="72">
+        <v>482</v>
+      </c>
+      <c r="AA13" s="72">
+        <v>0.2</v>
+      </c>
+      <c r="AB13" s="34">
+        <v>0.95</v>
+      </c>
+      <c r="AC13" s="34">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="14" spans="1:29" s="34" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="31">
         <v>12</v>
       </c>
       <c r="B14" s="38" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="C14" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="D14" s="29" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="E14" s="21" t="s">
         <v>52</v>
       </c>
       <c r="F14" s="21" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G14" s="9">
         <v>18</v>
@@ -3406,13 +3307,13 @@
         <v>20</v>
       </c>
       <c r="K14" s="9">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="L14" s="9">
         <v>540</v>
       </c>
       <c r="M14" s="22">
-        <v>6.26</v>
+        <v>8.73</v>
       </c>
       <c r="N14" s="35">
         <v>-1</v>
@@ -3427,7 +3328,7 @@
         <v>-1</v>
       </c>
       <c r="R14" s="22">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="S14" s="26">
         <v>0.92</v>
@@ -3439,39 +3340,32 @@
         <v>0.47</v>
       </c>
       <c r="V14" s="34">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="W14" s="34">
         <v>4</v>
       </c>
-      <c r="X14" s="24">
-        <v>360</v>
-      </c>
-      <c r="Y14" s="24">
+      <c r="X14" s="72">
+        <v>320</v>
+      </c>
+      <c r="Y14" s="72">
         <v>4</v>
       </c>
-      <c r="Z14" s="24">
-        <v>353</v>
-      </c>
-      <c r="AA14" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB14" t="s">
-        <v>61</v>
-      </c>
-      <c r="AC14" t="s">
-        <v>61</v>
-      </c>
-      <c r="AD14">
-        <v>8.3000000000000004E-2</v>
-      </c>
-      <c r="AE14">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="Z14" s="72">
+        <v>482</v>
+      </c>
+      <c r="AA14" s="72">
+        <v>0.2</v>
+      </c>
+      <c r="AB14" s="34">
+        <v>0.95</v>
+      </c>
+      <c r="AC14" s="34">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="15" spans="1:29" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:29" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
@@ -3499,34 +3393,34 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="C1" t="s">
+        <v>383</v>
+      </c>
+      <c r="D1" t="s">
+        <v>384</v>
+      </c>
+      <c r="E1" t="s">
+        <v>390</v>
+      </c>
+      <c r="F1" t="s">
+        <v>385</v>
+      </c>
+      <c r="G1" t="s">
+        <v>386</v>
+      </c>
+      <c r="H1" t="s">
+        <v>387</v>
+      </c>
+      <c r="I1" t="s">
+        <v>389</v>
+      </c>
+      <c r="J1" t="s">
         <v>388</v>
       </c>
-      <c r="D1" t="s">
-        <v>389</v>
-      </c>
-      <c r="E1" t="s">
-        <v>395</v>
-      </c>
-      <c r="F1" t="s">
-        <v>390</v>
-      </c>
-      <c r="G1" t="s">
-        <v>391</v>
-      </c>
-      <c r="H1" t="s">
-        <v>392</v>
-      </c>
-      <c r="I1" t="s">
-        <v>394</v>
-      </c>
-      <c r="J1" t="s">
-        <v>393</v>
-      </c>
       <c r="K1" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -3537,19 +3431,19 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="D2" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="E2" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="F2" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="G2" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="H2" t="s">
         <v>51</v>
@@ -3569,7 +3463,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="C3">
         <v>32711</v>
@@ -3604,7 +3498,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="C4">
         <v>32711</v>
@@ -3639,7 +3533,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="C5">
         <v>32711</v>
@@ -3685,22 +3579,22 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>372</v>
+      </c>
+      <c r="C1" t="s">
+        <v>373</v>
+      </c>
+      <c r="D1" t="s">
+        <v>374</v>
+      </c>
+      <c r="E1" t="s">
+        <v>375</v>
+      </c>
+      <c r="F1" t="s">
         <v>376</v>
       </c>
-      <c r="C1" t="s">
-        <v>377</v>
-      </c>
-      <c r="D1" t="s">
-        <v>378</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>379</v>
-      </c>
-      <c r="F1" t="s">
-        <v>380</v>
-      </c>
-      <c r="G1" t="s">
-        <v>383</v>
       </c>
       <c r="H1" s="13" t="s">
         <v>53</v>
@@ -3714,7 +3608,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="D2" t="s">
         <v>34</v>
@@ -3726,7 +3620,7 @@
         <v>34</v>
       </c>
       <c r="G2" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="H2" s="33" t="s">
         <v>4</v>
@@ -3737,7 +3631,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="C3">
         <v>18693</v>
@@ -3755,7 +3649,7 @@
         <v>79000</v>
       </c>
       <c r="H3" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
     </row>
   </sheetData>
@@ -3836,7 +3730,7 @@
         <v>0</v>
       </c>
       <c r="B3" s="50" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="C3" s="62" t="s">
         <v>6</v>
@@ -3862,7 +3756,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="50" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="C4" s="62" t="s">
         <v>6</v>
@@ -3888,7 +3782,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="50" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C5" s="62" t="s">
         <v>6</v>
@@ -3914,7 +3808,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="50" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C6" s="62" t="s">
         <v>6</v>
@@ -3940,7 +3834,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="50" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="C7" s="62" t="s">
         <v>6</v>
@@ -3966,7 +3860,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="50" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C8" s="62" t="s">
         <v>6</v>
@@ -3992,7 +3886,7 @@
         <v>6</v>
       </c>
       <c r="B9" s="50" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="C9" s="62" t="s">
         <v>6</v>
@@ -4018,7 +3912,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="50" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="C10" s="62" t="s">
         <v>6</v>
@@ -4044,7 +3938,7 @@
         <v>8</v>
       </c>
       <c r="B11" s="50" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C11" s="62" t="s">
         <v>6</v>
@@ -4070,7 +3964,7 @@
         <v>9</v>
       </c>
       <c r="B12" s="50" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="C12" s="62" t="s">
         <v>6</v>
@@ -4096,7 +3990,7 @@
         <v>10</v>
       </c>
       <c r="B13" s="50" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="C13" s="62" t="s">
         <v>6</v>
@@ -4122,7 +4016,7 @@
         <v>11</v>
       </c>
       <c r="B14" s="51" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="C14" s="62" t="s">
         <v>6</v>
@@ -4148,7 +4042,7 @@
         <v>12</v>
       </c>
       <c r="B15" s="51" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="C15" s="62" t="s">
         <v>6</v>
@@ -4174,7 +4068,7 @@
         <v>13</v>
       </c>
       <c r="B16" s="51" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="C16" s="62" t="s">
         <v>6</v>
@@ -4200,7 +4094,7 @@
         <v>14</v>
       </c>
       <c r="B17" s="51" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="C17" s="62" t="s">
         <v>6</v>
@@ -4226,7 +4120,7 @@
         <v>15</v>
       </c>
       <c r="B18" s="51" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="C18" s="62" t="s">
         <v>6</v>
@@ -4252,7 +4146,7 @@
         <v>16</v>
       </c>
       <c r="B19" s="51" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="C19" s="62" t="s">
         <v>6</v>
@@ -4278,7 +4172,7 @@
         <v>17</v>
       </c>
       <c r="B20" s="51" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="C20" s="62" t="s">
         <v>6</v>
@@ -4304,7 +4198,7 @@
         <v>18</v>
       </c>
       <c r="B21" s="51" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="C21" s="62" t="s">
         <v>6</v>
@@ -4330,7 +4224,7 @@
         <v>19</v>
       </c>
       <c r="B22" s="51" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="C22" s="62" t="s">
         <v>6</v>
@@ -4356,7 +4250,7 @@
         <v>20</v>
       </c>
       <c r="B23" s="51" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="C23" s="62" t="s">
         <v>6</v>
@@ -4382,7 +4276,7 @@
         <v>21</v>
       </c>
       <c r="B24" s="51" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="C24" s="62" t="s">
         <v>6</v>
@@ -4408,7 +4302,7 @@
         <v>22</v>
       </c>
       <c r="B25" s="51" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="C25" s="62" t="s">
         <v>6</v>
@@ -4434,7 +4328,7 @@
         <v>23</v>
       </c>
       <c r="B26" s="50" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C26" s="62" t="s">
         <v>13</v>
@@ -4460,7 +4354,7 @@
         <v>24</v>
       </c>
       <c r="B27" s="50" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="C27" s="62" t="s">
         <v>13</v>
@@ -4486,7 +4380,7 @@
         <v>25</v>
       </c>
       <c r="B28" s="50" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="C28" s="62" t="s">
         <v>13</v>
@@ -4512,7 +4406,7 @@
         <v>26</v>
       </c>
       <c r="B29" s="50" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="C29" s="62" t="s">
         <v>13</v>
@@ -4538,7 +4432,7 @@
         <v>27</v>
       </c>
       <c r="B30" s="50" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C30" s="62" t="s">
         <v>13</v>
@@ -4564,7 +4458,7 @@
         <v>28</v>
       </c>
       <c r="B31" s="50" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="C31" s="62" t="s">
         <v>13</v>
@@ -4590,7 +4484,7 @@
         <v>29</v>
       </c>
       <c r="B32" s="50" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C32" s="62" t="s">
         <v>13</v>
@@ -4616,7 +4510,7 @@
         <v>30</v>
       </c>
       <c r="B33" s="50" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="C33" s="62" t="s">
         <v>13</v>
@@ -4642,7 +4536,7 @@
         <v>31</v>
       </c>
       <c r="B34" s="50" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C34" s="62" t="s">
         <v>13</v>
@@ -4668,7 +4562,7 @@
         <v>32</v>
       </c>
       <c r="B35" s="50" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C35" s="62" t="s">
         <v>13</v>
@@ -4694,7 +4588,7 @@
         <v>33</v>
       </c>
       <c r="B36" s="50" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C36" s="62" t="s">
         <v>13</v>
@@ -4720,7 +4614,7 @@
         <v>34</v>
       </c>
       <c r="B37" s="50" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C37" s="62" t="s">
         <v>13</v>
@@ -4746,7 +4640,7 @@
         <v>35</v>
       </c>
       <c r="B38" s="50" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="C38" s="62" t="s">
         <v>13</v>
@@ -4772,7 +4666,7 @@
         <v>36</v>
       </c>
       <c r="B39" s="50" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="C39" s="62" t="s">
         <v>13</v>
@@ -4798,7 +4692,7 @@
         <v>37</v>
       </c>
       <c r="B40" s="50" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C40" s="62" t="s">
         <v>13</v>
@@ -4824,7 +4718,7 @@
         <v>38</v>
       </c>
       <c r="B41" s="50" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C41" s="62" t="s">
         <v>13</v>
@@ -4850,7 +4744,7 @@
         <v>39</v>
       </c>
       <c r="B42" s="50" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C42" s="62" t="s">
         <v>13</v>
@@ -4876,7 +4770,7 @@
         <v>40</v>
       </c>
       <c r="B43" s="50" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="C43" s="62" t="s">
         <v>13</v>
@@ -4902,7 +4796,7 @@
         <v>41</v>
       </c>
       <c r="B44" s="50" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C44" s="62" t="s">
         <v>13</v>
@@ -4928,7 +4822,7 @@
         <v>42</v>
       </c>
       <c r="B45" s="50" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="C45" s="62" t="s">
         <v>13</v>
@@ -4954,7 +4848,7 @@
         <v>43</v>
       </c>
       <c r="B46" s="50" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C46" s="62" t="s">
         <v>13</v>
@@ -4980,7 +4874,7 @@
         <v>44</v>
       </c>
       <c r="B47" s="50" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C47" s="62" t="s">
         <v>13</v>
@@ -5006,7 +4900,7 @@
         <v>45</v>
       </c>
       <c r="B48" s="50" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="C48" s="62" t="s">
         <v>13</v>
@@ -5032,7 +4926,7 @@
         <v>46</v>
       </c>
       <c r="B49" s="50" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="C49" s="62" t="s">
         <v>13</v>
@@ -5058,7 +4952,7 @@
         <v>47</v>
       </c>
       <c r="B50" s="50" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="C50" s="62" t="s">
         <v>14</v>
@@ -5084,7 +4978,7 @@
         <v>48</v>
       </c>
       <c r="B51" s="50" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C51" s="62" t="s">
         <v>14</v>
@@ -5110,7 +5004,7 @@
         <v>49</v>
       </c>
       <c r="B52" s="50" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C52" s="62" t="s">
         <v>14</v>
@@ -5136,7 +5030,7 @@
         <v>50</v>
       </c>
       <c r="B53" s="50" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="C53" s="62" t="s">
         <v>14</v>
@@ -5162,7 +5056,7 @@
         <v>51</v>
       </c>
       <c r="B54" s="50" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="C54" s="62" t="s">
         <v>14</v>
@@ -5188,7 +5082,7 @@
         <v>52</v>
       </c>
       <c r="B55" s="50" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="C55" s="62" t="s">
         <v>14</v>
@@ -5214,7 +5108,7 @@
         <v>53</v>
       </c>
       <c r="B56" s="50" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="C56" s="62" t="s">
         <v>14</v>
@@ -5240,7 +5134,7 @@
         <v>54</v>
       </c>
       <c r="B57" s="50" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C57" s="62" t="s">
         <v>14</v>
@@ -5266,7 +5160,7 @@
         <v>55</v>
       </c>
       <c r="B58" s="50" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C58" s="62" t="s">
         <v>14</v>
@@ -5292,7 +5186,7 @@
         <v>56</v>
       </c>
       <c r="B59" s="50" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C59" s="62" t="s">
         <v>14</v>
@@ -5318,7 +5212,7 @@
         <v>57</v>
       </c>
       <c r="B60" s="50" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C60" s="62" t="s">
         <v>14</v>
@@ -5344,7 +5238,7 @@
         <v>58</v>
       </c>
       <c r="B61" s="50" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C61" s="62" t="s">
         <v>14</v>
@@ -5370,7 +5264,7 @@
         <v>59</v>
       </c>
       <c r="B62" s="50" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C62" s="62" t="s">
         <v>14</v>
@@ -5396,7 +5290,7 @@
         <v>60</v>
       </c>
       <c r="B63" s="50" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C63" s="62" t="s">
         <v>14</v>
@@ -5422,7 +5316,7 @@
         <v>61</v>
       </c>
       <c r="B64" s="50" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C64" s="62" t="s">
         <v>14</v>
@@ -5448,7 +5342,7 @@
         <v>62</v>
       </c>
       <c r="B65" s="50" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C65" s="62" t="s">
         <v>14</v>
@@ -5474,7 +5368,7 @@
         <v>63</v>
       </c>
       <c r="B66" s="50" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C66" s="62" t="s">
         <v>14</v>
@@ -5500,7 +5394,7 @@
         <v>64</v>
       </c>
       <c r="B67" s="50" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C67" s="62" t="s">
         <v>14</v>
@@ -5526,7 +5420,7 @@
         <v>65</v>
       </c>
       <c r="B68" s="50" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C68" s="62" t="s">
         <v>14</v>
@@ -5552,7 +5446,7 @@
         <v>66</v>
       </c>
       <c r="B69" s="50" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C69" s="62" t="s">
         <v>14</v>
@@ -5578,7 +5472,7 @@
         <v>67</v>
       </c>
       <c r="B70" s="50" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="C70" s="62" t="s">
         <v>14</v>
@@ -5604,7 +5498,7 @@
         <v>68</v>
       </c>
       <c r="B71" s="50" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C71" s="62" t="s">
         <v>14</v>
@@ -5630,7 +5524,7 @@
         <v>69</v>
       </c>
       <c r="B72" s="50" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C72" s="62" t="s">
         <v>14</v>
@@ -5656,7 +5550,7 @@
         <v>70</v>
       </c>
       <c r="B73" s="50" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="C73" s="62" t="s">
         <v>14</v>
@@ -5682,7 +5576,7 @@
         <v>71</v>
       </c>
       <c r="B74" s="50" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="C74" s="62" t="s">
         <v>15</v>
@@ -5708,7 +5602,7 @@
         <v>72</v>
       </c>
       <c r="B75" s="50" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C75" s="62" t="s">
         <v>15</v>
@@ -5734,7 +5628,7 @@
         <v>73</v>
       </c>
       <c r="B76" s="50" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C76" s="62" t="s">
         <v>15</v>
@@ -5760,7 +5654,7 @@
         <v>74</v>
       </c>
       <c r="B77" s="50" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C77" s="62" t="s">
         <v>15</v>
@@ -5786,7 +5680,7 @@
         <v>75</v>
       </c>
       <c r="B78" s="50" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C78" s="62" t="s">
         <v>15</v>
@@ -5812,7 +5706,7 @@
         <v>76</v>
       </c>
       <c r="B79" s="50" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C79" s="62" t="s">
         <v>15</v>
@@ -5838,7 +5732,7 @@
         <v>77</v>
       </c>
       <c r="B80" s="50" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C80" s="62" t="s">
         <v>15</v>
@@ -5864,7 +5758,7 @@
         <v>78</v>
       </c>
       <c r="B81" s="50" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C81" s="62" t="s">
         <v>15</v>
@@ -5890,7 +5784,7 @@
         <v>79</v>
       </c>
       <c r="B82" s="50" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C82" s="62" t="s">
         <v>15</v>
@@ -5916,7 +5810,7 @@
         <v>80</v>
       </c>
       <c r="B83" s="50" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="C83" s="62" t="s">
         <v>15</v>
@@ -5942,7 +5836,7 @@
         <v>81</v>
       </c>
       <c r="B84" s="50" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C84" s="62" t="s">
         <v>15</v>
@@ -5968,7 +5862,7 @@
         <v>82</v>
       </c>
       <c r="B85" s="50" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="C85" s="62" t="s">
         <v>15</v>
@@ -5994,7 +5888,7 @@
         <v>83</v>
       </c>
       <c r="B86" s="50" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C86" s="62" t="s">
         <v>15</v>
@@ -6020,7 +5914,7 @@
         <v>84</v>
       </c>
       <c r="B87" s="50" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="C87" s="62" t="s">
         <v>15</v>
@@ -6046,7 +5940,7 @@
         <v>85</v>
       </c>
       <c r="B88" s="50" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="C88" s="62" t="s">
         <v>15</v>
@@ -6072,7 +5966,7 @@
         <v>86</v>
       </c>
       <c r="B89" s="50" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="C89" s="62" t="s">
         <v>15</v>
@@ -6098,7 +5992,7 @@
         <v>87</v>
       </c>
       <c r="B90" s="50" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="C90" s="62" t="s">
         <v>15</v>
@@ -6124,7 +6018,7 @@
         <v>88</v>
       </c>
       <c r="B91" s="50" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="C91" s="62" t="s">
         <v>15</v>
@@ -6150,7 +6044,7 @@
         <v>89</v>
       </c>
       <c r="B92" s="50" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="C92" s="62" t="s">
         <v>15</v>
@@ -6176,7 +6070,7 @@
         <v>90</v>
       </c>
       <c r="B93" s="50" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="C93" s="62" t="s">
         <v>15</v>
@@ -6202,7 +6096,7 @@
         <v>91</v>
       </c>
       <c r="B94" s="50" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="C94" s="62" t="s">
         <v>15</v>
@@ -6228,7 +6122,7 @@
         <v>92</v>
       </c>
       <c r="B95" s="50" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="C95" s="62" t="s">
         <v>15</v>
@@ -6254,7 +6148,7 @@
         <v>93</v>
       </c>
       <c r="B96" s="50" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="C96" s="62" t="s">
         <v>15</v>
@@ -6280,10 +6174,10 @@
         <v>94</v>
       </c>
       <c r="B97" s="48" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C97" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D97" s="46" t="s">
         <v>5</v>
@@ -6306,10 +6200,10 @@
         <v>95</v>
       </c>
       <c r="B98" s="48" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C98" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D98" s="46" t="s">
         <v>5</v>
@@ -6332,10 +6226,10 @@
         <v>96</v>
       </c>
       <c r="B99" s="48" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C99" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D99" s="46" t="s">
         <v>5</v>
@@ -6358,10 +6252,10 @@
         <v>97</v>
       </c>
       <c r="B100" s="48" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C100" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D100" s="46" t="s">
         <v>5</v>
@@ -6384,10 +6278,10 @@
         <v>98</v>
       </c>
       <c r="B101" s="48" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C101" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D101" s="46" t="s">
         <v>5</v>
@@ -6410,10 +6304,10 @@
         <v>99</v>
       </c>
       <c r="B102" s="48" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C102" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D102" s="46" t="s">
         <v>5</v>
@@ -6436,10 +6330,10 @@
         <v>100</v>
       </c>
       <c r="B103" s="48" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C103" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D103" s="46" t="s">
         <v>5</v>
@@ -6462,10 +6356,10 @@
         <v>101</v>
       </c>
       <c r="B104" s="48" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C104" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D104" s="46" t="s">
         <v>5</v>
@@ -6488,10 +6382,10 @@
         <v>102</v>
       </c>
       <c r="B105" s="48" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C105" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D105" s="46" t="s">
         <v>5</v>
@@ -6514,10 +6408,10 @@
         <v>103</v>
       </c>
       <c r="B106" s="48" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C106" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D106" s="46" t="s">
         <v>5</v>
@@ -6540,10 +6434,10 @@
         <v>104</v>
       </c>
       <c r="B107" s="48" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C107" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D107" s="46" t="s">
         <v>5</v>
@@ -6566,10 +6460,10 @@
         <v>105</v>
       </c>
       <c r="B108" s="48" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C108" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D108" s="46" t="s">
         <v>5</v>
@@ -6592,10 +6486,10 @@
         <v>106</v>
       </c>
       <c r="B109" s="48" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C109" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D109" s="46" t="s">
         <v>5</v>
@@ -6618,10 +6512,10 @@
         <v>107</v>
       </c>
       <c r="B110" s="48" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C110" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D110" s="46" t="s">
         <v>5</v>
@@ -6644,10 +6538,10 @@
         <v>108</v>
       </c>
       <c r="B111" s="48" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C111" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D111" s="46" t="s">
         <v>5</v>
@@ -6670,10 +6564,10 @@
         <v>109</v>
       </c>
       <c r="B112" s="48" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C112" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D112" s="46" t="s">
         <v>5</v>
@@ -6696,10 +6590,10 @@
         <v>110</v>
       </c>
       <c r="B113" s="48" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C113" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D113" s="46" t="s">
         <v>5</v>
@@ -6722,10 +6616,10 @@
         <v>111</v>
       </c>
       <c r="B114" s="48" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C114" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D114" s="46" t="s">
         <v>5</v>
@@ -6748,10 +6642,10 @@
         <v>112</v>
       </c>
       <c r="B115" s="48" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C115" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D115" s="46" t="s">
         <v>5</v>
@@ -6774,10 +6668,10 @@
         <v>113</v>
       </c>
       <c r="B116" s="48" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C116" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D116" s="46" t="s">
         <v>5</v>
@@ -6800,10 +6694,10 @@
         <v>114</v>
       </c>
       <c r="B117" s="48" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C117" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D117" s="46" t="s">
         <v>5</v>
@@ -6826,10 +6720,10 @@
         <v>115</v>
       </c>
       <c r="B118" s="48" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C118" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D118" s="46" t="s">
         <v>5</v>
@@ -6852,10 +6746,10 @@
         <v>116</v>
       </c>
       <c r="B119" s="48" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C119" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D119" s="46" t="s">
         <v>5</v>
@@ -6878,10 +6772,10 @@
         <v>117</v>
       </c>
       <c r="B120" s="48" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C120" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D120" s="46" t="s">
         <v>5</v>
@@ -6904,10 +6798,10 @@
         <v>118</v>
       </c>
       <c r="B121" s="48" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C121" s="62" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D121" s="46" t="s">
         <v>5</v>
@@ -6930,10 +6824,10 @@
         <v>119</v>
       </c>
       <c r="B122" s="48" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C122" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D122" s="46" t="s">
         <v>5</v>
@@ -6956,10 +6850,10 @@
         <v>120</v>
       </c>
       <c r="B123" s="48" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C123" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D123" s="46" t="s">
         <v>5</v>
@@ -6982,10 +6876,10 @@
         <v>121</v>
       </c>
       <c r="B124" s="48" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C124" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D124" s="46" t="s">
         <v>5</v>
@@ -7008,10 +6902,10 @@
         <v>122</v>
       </c>
       <c r="B125" s="48" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C125" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D125" s="46" t="s">
         <v>5</v>
@@ -7034,10 +6928,10 @@
         <v>123</v>
       </c>
       <c r="B126" s="48" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C126" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D126" s="46" t="s">
         <v>5</v>
@@ -7060,10 +6954,10 @@
         <v>124</v>
       </c>
       <c r="B127" s="48" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C127" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D127" s="46" t="s">
         <v>5</v>
@@ -7086,10 +6980,10 @@
         <v>125</v>
       </c>
       <c r="B128" s="48" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C128" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D128" s="46" t="s">
         <v>5</v>
@@ -7112,10 +7006,10 @@
         <v>126</v>
       </c>
       <c r="B129" s="48" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C129" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D129" s="46" t="s">
         <v>5</v>
@@ -7138,10 +7032,10 @@
         <v>127</v>
       </c>
       <c r="B130" s="48" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C130" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D130" s="46" t="s">
         <v>5</v>
@@ -7164,10 +7058,10 @@
         <v>128</v>
       </c>
       <c r="B131" s="48" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C131" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D131" s="46" t="s">
         <v>5</v>
@@ -7190,10 +7084,10 @@
         <v>129</v>
       </c>
       <c r="B132" s="48" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C132" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D132" s="46" t="s">
         <v>5</v>
@@ -7216,10 +7110,10 @@
         <v>130</v>
       </c>
       <c r="B133" s="48" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C133" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D133" s="46" t="s">
         <v>5</v>
@@ -7242,10 +7136,10 @@
         <v>131</v>
       </c>
       <c r="B134" s="48" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C134" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D134" s="46" t="s">
         <v>5</v>
@@ -7268,10 +7162,10 @@
         <v>132</v>
       </c>
       <c r="B135" s="48" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C135" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D135" s="46" t="s">
         <v>5</v>
@@ -7294,10 +7188,10 @@
         <v>133</v>
       </c>
       <c r="B136" s="48" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C136" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D136" s="46" t="s">
         <v>5</v>
@@ -7320,10 +7214,10 @@
         <v>134</v>
       </c>
       <c r="B137" s="49" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C137" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D137" s="46" t="s">
         <v>5</v>
@@ -7346,10 +7240,10 @@
         <v>135</v>
       </c>
       <c r="B138" s="49" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C138" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D138" s="46" t="s">
         <v>5</v>
@@ -7372,10 +7266,10 @@
         <v>136</v>
       </c>
       <c r="B139" s="49" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C139" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D139" s="46" t="s">
         <v>5</v>
@@ -7398,10 +7292,10 @@
         <v>137</v>
       </c>
       <c r="B140" s="49" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C140" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D140" s="46" t="s">
         <v>5</v>
@@ -7424,10 +7318,10 @@
         <v>138</v>
       </c>
       <c r="B141" s="49" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C141" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D141" s="46" t="s">
         <v>5</v>
@@ -7450,10 +7344,10 @@
         <v>139</v>
       </c>
       <c r="B142" s="49" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C142" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D142" s="46" t="s">
         <v>5</v>
@@ -7476,10 +7370,10 @@
         <v>140</v>
       </c>
       <c r="B143" s="49" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C143" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D143" s="46" t="s">
         <v>5</v>
@@ -7502,10 +7396,10 @@
         <v>141</v>
       </c>
       <c r="B144" s="49" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C144" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D144" s="46" t="s">
         <v>5</v>
@@ -7528,10 +7422,10 @@
         <v>142</v>
       </c>
       <c r="B145" s="49" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C145" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D145" s="46" t="s">
         <v>5</v>
@@ -7554,10 +7448,10 @@
         <v>143</v>
       </c>
       <c r="B146" s="49" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C146" s="62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D146" s="46" t="s">
         <v>5</v>
@@ -7580,10 +7474,10 @@
         <v>144</v>
       </c>
       <c r="B147" s="49" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C147" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D147" s="46" t="s">
         <v>5</v>
@@ -7606,10 +7500,10 @@
         <v>145</v>
       </c>
       <c r="B148" s="49" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C148" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D148" s="46" t="s">
         <v>5</v>
@@ -7632,10 +7526,10 @@
         <v>146</v>
       </c>
       <c r="B149" s="49" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C149" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D149" s="46" t="s">
         <v>5</v>
@@ -7658,10 +7552,10 @@
         <v>147</v>
       </c>
       <c r="B150" s="49" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C150" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D150" s="46" t="s">
         <v>5</v>
@@ -7684,10 +7578,10 @@
         <v>148</v>
       </c>
       <c r="B151" s="49" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C151" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D151" s="46" t="s">
         <v>5</v>
@@ -7710,10 +7604,10 @@
         <v>149</v>
       </c>
       <c r="B152" s="49" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C152" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D152" s="46" t="s">
         <v>5</v>
@@ -7736,10 +7630,10 @@
         <v>150</v>
       </c>
       <c r="B153" s="49" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C153" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D153" s="46" t="s">
         <v>5</v>
@@ -7762,10 +7656,10 @@
         <v>151</v>
       </c>
       <c r="B154" s="49" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C154" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D154" s="46" t="s">
         <v>5</v>
@@ -7788,10 +7682,10 @@
         <v>152</v>
       </c>
       <c r="B155" s="49" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C155" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D155" s="46" t="s">
         <v>5</v>
@@ -7814,10 +7708,10 @@
         <v>153</v>
       </c>
       <c r="B156" s="49" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C156" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D156" s="46" t="s">
         <v>5</v>
@@ -7840,10 +7734,10 @@
         <v>154</v>
       </c>
       <c r="B157" s="49" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C157" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D157" s="46" t="s">
         <v>5</v>
@@ -7866,10 +7760,10 @@
         <v>155</v>
       </c>
       <c r="B158" s="49" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C158" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D158" s="46" t="s">
         <v>5</v>
@@ -7892,10 +7786,10 @@
         <v>156</v>
       </c>
       <c r="B159" s="49" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C159" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D159" s="46" t="s">
         <v>5</v>
@@ -7918,10 +7812,10 @@
         <v>157</v>
       </c>
       <c r="B160" s="49" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C160" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D160" s="46" t="s">
         <v>5</v>
@@ -7944,10 +7838,10 @@
         <v>158</v>
       </c>
       <c r="B161" s="49" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C161" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D161" s="46" t="s">
         <v>5</v>
@@ -7970,10 +7864,10 @@
         <v>159</v>
       </c>
       <c r="B162" s="49" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C162" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D162" s="46" t="s">
         <v>5</v>
@@ -7996,10 +7890,10 @@
         <v>160</v>
       </c>
       <c r="B163" s="49" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C163" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D163" s="46" t="s">
         <v>5</v>
@@ -8022,10 +7916,10 @@
         <v>161</v>
       </c>
       <c r="B164" s="49" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C164" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D164" s="46" t="s">
         <v>5</v>
@@ -8048,10 +7942,10 @@
         <v>162</v>
       </c>
       <c r="B165" s="49" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C165" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D165" s="46" t="s">
         <v>5</v>
@@ -8074,10 +7968,10 @@
         <v>163</v>
       </c>
       <c r="B166" s="49" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C166" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D166" s="46" t="s">
         <v>5</v>
@@ -8100,10 +7994,10 @@
         <v>164</v>
       </c>
       <c r="B167" s="49" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C167" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D167" s="46" t="s">
         <v>5</v>
@@ -8126,10 +8020,10 @@
         <v>165</v>
       </c>
       <c r="B168" s="49" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C168" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D168" s="46" t="s">
         <v>5</v>
@@ -8152,10 +8046,10 @@
         <v>166</v>
       </c>
       <c r="B169" s="49" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C169" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D169" s="46" t="s">
         <v>5</v>
@@ -8178,10 +8072,10 @@
         <v>167</v>
       </c>
       <c r="B170" s="49" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C170" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D170" s="46" t="s">
         <v>5</v>
@@ -8204,10 +8098,10 @@
         <v>168</v>
       </c>
       <c r="B171" s="49" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C171" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D171" s="46" t="s">
         <v>5</v>
@@ -8230,10 +8124,10 @@
         <v>169</v>
       </c>
       <c r="B172" s="49" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C172" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D172" s="46" t="s">
         <v>5</v>
@@ -8256,10 +8150,10 @@
         <v>170</v>
       </c>
       <c r="B173" s="49" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="C173" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D173" s="46" t="s">
         <v>5</v>
@@ -8282,10 +8176,10 @@
         <v>171</v>
       </c>
       <c r="B174" s="49" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C174" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D174" s="46" t="s">
         <v>5</v>
@@ -8308,10 +8202,10 @@
         <v>172</v>
       </c>
       <c r="B175" s="49" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C175" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D175" s="46" t="s">
         <v>5</v>
@@ -8334,10 +8228,10 @@
         <v>173</v>
       </c>
       <c r="B176" s="49" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C176" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D176" s="46" t="s">
         <v>5</v>
@@ -8360,10 +8254,10 @@
         <v>174</v>
       </c>
       <c r="B177" s="49" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C177" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D177" s="46" t="s">
         <v>5</v>
@@ -8386,10 +8280,10 @@
         <v>175</v>
       </c>
       <c r="B178" s="49" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C178" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D178" s="46" t="s">
         <v>5</v>
@@ -8412,10 +8306,10 @@
         <v>176</v>
       </c>
       <c r="B179" s="49" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C179" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D179" s="46" t="s">
         <v>5</v>
@@ -8438,10 +8332,10 @@
         <v>177</v>
       </c>
       <c r="B180" s="49" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C180" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D180" s="46" t="s">
         <v>5</v>
@@ -8464,10 +8358,10 @@
         <v>178</v>
       </c>
       <c r="B181" s="49" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C181" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D181" s="46" t="s">
         <v>5</v>
@@ -8490,10 +8384,10 @@
         <v>179</v>
       </c>
       <c r="B182" s="49" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C182" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D182" s="46" t="s">
         <v>5</v>
@@ -8516,10 +8410,10 @@
         <v>180</v>
       </c>
       <c r="B183" s="49" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C183" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D183" s="46" t="s">
         <v>5</v>
@@ -8542,10 +8436,10 @@
         <v>181</v>
       </c>
       <c r="B184" s="49" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C184" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D184" s="46" t="s">
         <v>5</v>
@@ -8568,10 +8462,10 @@
         <v>182</v>
       </c>
       <c r="B185" s="49" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C185" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D185" s="46" t="s">
         <v>5</v>
@@ -8594,10 +8488,10 @@
         <v>183</v>
       </c>
       <c r="B186" s="49" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C186" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D186" s="46" t="s">
         <v>5</v>
@@ -8620,10 +8514,10 @@
         <v>184</v>
       </c>
       <c r="B187" s="49" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C187" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D187" s="46" t="s">
         <v>5</v>
@@ -8646,10 +8540,10 @@
         <v>185</v>
       </c>
       <c r="B188" s="49" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C188" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D188" s="46" t="s">
         <v>5</v>
@@ -8672,10 +8566,10 @@
         <v>186</v>
       </c>
       <c r="B189" s="49" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C189" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D189" s="46" t="s">
         <v>5</v>
@@ -8698,10 +8592,10 @@
         <v>187</v>
       </c>
       <c r="B190" s="49" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="C190" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D190" s="46" t="s">
         <v>5</v>
@@ -8724,10 +8618,10 @@
         <v>188</v>
       </c>
       <c r="B191" s="49" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="C191" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D191" s="46" t="s">
         <v>5</v>
@@ -8750,10 +8644,10 @@
         <v>189</v>
       </c>
       <c r="B192" s="49" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="C192" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D192" s="46" t="s">
         <v>5</v>
@@ -8776,10 +8670,10 @@
         <v>190</v>
       </c>
       <c r="B193" s="49" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="C193" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D193" s="46" t="s">
         <v>5</v>
@@ -8802,10 +8696,10 @@
         <v>191</v>
       </c>
       <c r="B194" s="49" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="C194" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D194" s="46" t="s">
         <v>5</v>
@@ -8828,10 +8722,10 @@
         <v>192</v>
       </c>
       <c r="B195" s="49" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="C195" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D195" s="46" t="s">
         <v>5</v>
@@ -8854,10 +8748,10 @@
         <v>193</v>
       </c>
       <c r="B196" s="49" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="C196" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D196" s="46" t="s">
         <v>5</v>
@@ -8880,10 +8774,10 @@
         <v>194</v>
       </c>
       <c r="B197" s="50" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="C197" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D197" s="46" t="s">
         <v>5</v>
@@ -8906,10 +8800,10 @@
         <v>195</v>
       </c>
       <c r="B198" s="50" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="C198" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D198" s="46" t="s">
         <v>5</v>
@@ -8932,10 +8826,10 @@
         <v>196</v>
       </c>
       <c r="B199" s="50" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="C199" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D199" s="46" t="s">
         <v>5</v>
@@ -8958,10 +8852,10 @@
         <v>197</v>
       </c>
       <c r="B200" s="50" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="C200" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D200" s="46" t="s">
         <v>5</v>
@@ -8984,10 +8878,10 @@
         <v>198</v>
       </c>
       <c r="B201" s="50" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="C201" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D201" s="46" t="s">
         <v>5</v>
@@ -9010,10 +8904,10 @@
         <v>199</v>
       </c>
       <c r="B202" s="50" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="C202" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D202" s="46" t="s">
         <v>5</v>
@@ -9036,10 +8930,10 @@
         <v>200</v>
       </c>
       <c r="B203" s="50" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C203" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D203" s="46" t="s">
         <v>5</v>
@@ -9062,10 +8956,10 @@
         <v>201</v>
       </c>
       <c r="B204" s="50" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="C204" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D204" s="46" t="s">
         <v>5</v>
@@ -9088,10 +8982,10 @@
         <v>202</v>
       </c>
       <c r="B205" s="50" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="C205" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D205" s="46" t="s">
         <v>5</v>
@@ -9114,10 +9008,10 @@
         <v>203</v>
       </c>
       <c r="B206" s="50" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C206" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D206" s="46" t="s">
         <v>5</v>
@@ -9140,10 +9034,10 @@
         <v>204</v>
       </c>
       <c r="B207" s="50" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="C207" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D207" s="46" t="s">
         <v>5</v>
@@ -9166,10 +9060,10 @@
         <v>205</v>
       </c>
       <c r="B208" s="50" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="C208" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D208" s="46" t="s">
         <v>5</v>
@@ -9192,10 +9086,10 @@
         <v>206</v>
       </c>
       <c r="B209" s="50" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="C209" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D209" s="46" t="s">
         <v>5</v>
@@ -9218,10 +9112,10 @@
         <v>207</v>
       </c>
       <c r="B210" s="50" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C210" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D210" s="46" t="s">
         <v>5</v>
@@ -9244,10 +9138,10 @@
         <v>208</v>
       </c>
       <c r="B211" s="50" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="C211" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D211" s="46" t="s">
         <v>5</v>
@@ -9270,10 +9164,10 @@
         <v>209</v>
       </c>
       <c r="B212" s="50" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C212" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D212" s="46" t="s">
         <v>5</v>
@@ -9296,10 +9190,10 @@
         <v>210</v>
       </c>
       <c r="B213" s="50" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C213" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D213" s="46" t="s">
         <v>5</v>
@@ -9322,10 +9216,10 @@
         <v>211</v>
       </c>
       <c r="B214" s="50" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="C214" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D214" s="46" t="s">
         <v>5</v>
@@ -9348,10 +9242,10 @@
         <v>212</v>
       </c>
       <c r="B215" s="50" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="C215" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D215" s="46" t="s">
         <v>5</v>
@@ -9374,10 +9268,10 @@
         <v>213</v>
       </c>
       <c r="B216" s="50" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="C216" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D216" s="46" t="s">
         <v>5</v>
@@ -9400,10 +9294,10 @@
         <v>214</v>
       </c>
       <c r="B217" s="50" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="C217" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D217" s="46" t="s">
         <v>5</v>
@@ -9426,10 +9320,10 @@
         <v>215</v>
       </c>
       <c r="B218" s="50" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C218" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D218" s="46" t="s">
         <v>5</v>
@@ -9452,10 +9346,10 @@
         <v>216</v>
       </c>
       <c r="B219" s="50" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="C219" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D219" s="46" t="s">
         <v>5</v>
@@ -9478,10 +9372,10 @@
         <v>217</v>
       </c>
       <c r="B220" s="50" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="C220" s="62" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D220" s="46" t="s">
         <v>5</v>
@@ -9504,10 +9398,10 @@
         <v>218</v>
       </c>
       <c r="B221" s="50" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="C221" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D221" s="46" t="s">
         <v>5</v>
@@ -9530,10 +9424,10 @@
         <v>219</v>
       </c>
       <c r="B222" s="50" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="C222" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D222" s="46" t="s">
         <v>5</v>
@@ -9556,10 +9450,10 @@
         <v>220</v>
       </c>
       <c r="B223" s="50" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="C223" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D223" s="46" t="s">
         <v>5</v>
@@ -9582,10 +9476,10 @@
         <v>221</v>
       </c>
       <c r="B224" s="50" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="C224" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D224" s="46" t="s">
         <v>5</v>
@@ -9608,10 +9502,10 @@
         <v>222</v>
       </c>
       <c r="B225" s="50" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="C225" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D225" s="46" t="s">
         <v>5</v>
@@ -9634,10 +9528,10 @@
         <v>223</v>
       </c>
       <c r="B226" s="50" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="C226" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D226" s="46" t="s">
         <v>5</v>
@@ -9660,10 +9554,10 @@
         <v>224</v>
       </c>
       <c r="B227" s="50" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="C227" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D227" s="46" t="s">
         <v>5</v>
@@ -9686,10 +9580,10 @@
         <v>225</v>
       </c>
       <c r="B228" s="50" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="C228" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D228" s="46" t="s">
         <v>5</v>
@@ -9712,10 +9606,10 @@
         <v>226</v>
       </c>
       <c r="B229" s="50" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="C229" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D229" s="46" t="s">
         <v>5</v>
@@ -9738,10 +9632,10 @@
         <v>227</v>
       </c>
       <c r="B230" s="50" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="C230" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D230" s="46" t="s">
         <v>5</v>
@@ -9764,10 +9658,10 @@
         <v>228</v>
       </c>
       <c r="B231" s="50" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="C231" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D231" s="46" t="s">
         <v>5</v>
@@ -9790,10 +9684,10 @@
         <v>229</v>
       </c>
       <c r="B232" s="50" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="C232" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D232" s="46" t="s">
         <v>5</v>
@@ -9816,10 +9710,10 @@
         <v>230</v>
       </c>
       <c r="B233" s="50" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="C233" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D233" s="46" t="s">
         <v>5</v>
@@ -9842,10 +9736,10 @@
         <v>231</v>
       </c>
       <c r="B234" s="50" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="C234" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D234" s="46" t="s">
         <v>5</v>
@@ -9868,10 +9762,10 @@
         <v>232</v>
       </c>
       <c r="B235" s="50" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="C235" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D235" s="46" t="s">
         <v>5</v>
@@ -9894,10 +9788,10 @@
         <v>233</v>
       </c>
       <c r="B236" s="50" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="C236" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D236" s="46" t="s">
         <v>5</v>
@@ -9920,10 +9814,10 @@
         <v>234</v>
       </c>
       <c r="B237" s="50" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C237" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D237" s="46" t="s">
         <v>5</v>
@@ -9946,10 +9840,10 @@
         <v>235</v>
       </c>
       <c r="B238" s="50" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="C238" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D238" s="46" t="s">
         <v>5</v>
@@ -9972,10 +9866,10 @@
         <v>236</v>
       </c>
       <c r="B239" s="50" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="C239" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D239" s="46" t="s">
         <v>5</v>
@@ -9998,10 +9892,10 @@
         <v>237</v>
       </c>
       <c r="B240" s="50" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C240" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D240" s="46" t="s">
         <v>5</v>
@@ -10024,10 +9918,10 @@
         <v>238</v>
       </c>
       <c r="B241" s="50" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="C241" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D241" s="46" t="s">
         <v>5</v>
@@ -10050,10 +9944,10 @@
         <v>239</v>
       </c>
       <c r="B242" s="50" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="C242" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D242" s="46" t="s">
         <v>5</v>
@@ -10076,10 +9970,10 @@
         <v>240</v>
       </c>
       <c r="B243" s="50" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="C243" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D243" s="46" t="s">
         <v>5</v>
@@ -10102,10 +9996,10 @@
         <v>241</v>
       </c>
       <c r="B244" s="50" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="C244" s="62" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D244" s="46" t="s">
         <v>5</v>
@@ -10128,10 +10022,10 @@
         <v>242</v>
       </c>
       <c r="B245" s="50" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="C245" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D245" s="46" t="s">
         <v>5</v>
@@ -10154,10 +10048,10 @@
         <v>243</v>
       </c>
       <c r="B246" s="50" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="C246" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D246" s="46" t="s">
         <v>5</v>
@@ -10180,10 +10074,10 @@
         <v>244</v>
       </c>
       <c r="B247" s="50" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="C247" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D247" s="46" t="s">
         <v>5</v>
@@ -10206,10 +10100,10 @@
         <v>245</v>
       </c>
       <c r="B248" s="50" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="C248" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D248" s="46" t="s">
         <v>5</v>
@@ -10232,10 +10126,10 @@
         <v>246</v>
       </c>
       <c r="B249" s="50" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="C249" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D249" s="46" t="s">
         <v>5</v>
@@ -10258,10 +10152,10 @@
         <v>247</v>
       </c>
       <c r="B250" s="50" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="C250" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D250" s="46" t="s">
         <v>5</v>
@@ -10284,10 +10178,10 @@
         <v>248</v>
       </c>
       <c r="B251" s="50" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="C251" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D251" s="46" t="s">
         <v>5</v>
@@ -10310,10 +10204,10 @@
         <v>249</v>
       </c>
       <c r="B252" s="50" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="C252" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D252" s="46" t="s">
         <v>5</v>
@@ -10336,10 +10230,10 @@
         <v>250</v>
       </c>
       <c r="B253" s="50" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="C253" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D253" s="46" t="s">
         <v>5</v>
@@ -10362,10 +10256,10 @@
         <v>251</v>
       </c>
       <c r="B254" s="50" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="C254" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D254" s="46" t="s">
         <v>5</v>
@@ -10388,10 +10282,10 @@
         <v>252</v>
       </c>
       <c r="B255" s="50" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="C255" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D255" s="46" t="s">
         <v>5</v>
@@ -10414,10 +10308,10 @@
         <v>253</v>
       </c>
       <c r="B256" s="50" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="C256" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D256" s="46" t="s">
         <v>5</v>
@@ -10440,10 +10334,10 @@
         <v>254</v>
       </c>
       <c r="B257" s="50" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="C257" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D257" s="46" t="s">
         <v>5</v>
@@ -10466,10 +10360,10 @@
         <v>255</v>
       </c>
       <c r="B258" s="50" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="C258" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D258" s="46" t="s">
         <v>5</v>
@@ -10492,10 +10386,10 @@
         <v>256</v>
       </c>
       <c r="B259" s="50" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="C259" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D259" s="46" t="s">
         <v>5</v>
@@ -10518,10 +10412,10 @@
         <v>257</v>
       </c>
       <c r="B260" s="50" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="C260" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D260" s="46" t="s">
         <v>5</v>
@@ -10544,10 +10438,10 @@
         <v>258</v>
       </c>
       <c r="B261" s="50" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="C261" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D261" s="46" t="s">
         <v>5</v>
@@ -10570,10 +10464,10 @@
         <v>259</v>
       </c>
       <c r="B262" s="50" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="C262" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D262" s="46" t="s">
         <v>5</v>
@@ -10596,10 +10490,10 @@
         <v>260</v>
       </c>
       <c r="B263" s="50" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="C263" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D263" s="46" t="s">
         <v>5</v>
@@ -10622,10 +10516,10 @@
         <v>261</v>
       </c>
       <c r="B264" s="50" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="C264" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D264" s="46" t="s">
         <v>5</v>
@@ -10648,10 +10542,10 @@
         <v>262</v>
       </c>
       <c r="B265" s="50" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="C265" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D265" s="46" t="s">
         <v>5</v>
@@ -10674,10 +10568,10 @@
         <v>263</v>
       </c>
       <c r="B266" s="50" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="C266" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D266" s="46" t="s">
         <v>5</v>
@@ -10700,10 +10594,10 @@
         <v>264</v>
       </c>
       <c r="B267" s="50" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="C267" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D267" s="46" t="s">
         <v>5</v>
@@ -10726,10 +10620,10 @@
         <v>265</v>
       </c>
       <c r="B268" s="50" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="C268" s="62" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D268" s="46" t="s">
         <v>5</v>
@@ -10752,10 +10646,10 @@
         <v>266</v>
       </c>
       <c r="B269" s="50" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="C269" s="62" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D269" s="46" t="s">
         <v>5</v>
@@ -10778,10 +10672,10 @@
         <v>267</v>
       </c>
       <c r="B270" s="50" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="C270" s="62" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D270" s="46" t="s">
         <v>5</v>
@@ -10804,10 +10698,10 @@
         <v>268</v>
       </c>
       <c r="B271" s="50" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="C271" s="62" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D271" s="46" t="s">
         <v>5</v>
@@ -10830,10 +10724,10 @@
         <v>269</v>
       </c>
       <c r="B272" s="50" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="C272" s="62" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D272" s="46" t="s">
         <v>5</v>
@@ -10856,10 +10750,10 @@
         <v>270</v>
       </c>
       <c r="B273" s="50" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="C273" s="62" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D273" s="46" t="s">
         <v>5</v>
@@ -10882,10 +10776,10 @@
         <v>271</v>
       </c>
       <c r="B274" s="50" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="C274" s="62" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D274" s="46" t="s">
         <v>5</v>
@@ -10908,10 +10802,10 @@
         <v>272</v>
       </c>
       <c r="B275" s="50" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="C275" s="62" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D275" s="46" t="s">
         <v>5</v>
@@ -10934,10 +10828,10 @@
         <v>273</v>
       </c>
       <c r="B276" s="50" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="C276" s="62" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D276" s="46" t="s">
         <v>5</v>
@@ -10960,10 +10854,10 @@
         <v>274</v>
       </c>
       <c r="B277" s="50" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="C277" s="62" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D277" s="46" t="s">
         <v>5</v>
@@ -10986,10 +10880,10 @@
         <v>275</v>
       </c>
       <c r="B278" s="50" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="C278" s="62" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D278" s="46" t="s">
         <v>5</v>
@@ -11012,10 +10906,10 @@
         <v>276</v>
       </c>
       <c r="B279" s="50" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="C279" s="62" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D279" s="46" t="s">
         <v>5</v>
@@ -11038,10 +10932,10 @@
         <v>277</v>
       </c>
       <c r="B280" s="50" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="C280" s="62" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D280" s="46" t="s">
         <v>5</v>
@@ -11064,10 +10958,10 @@
         <v>278</v>
       </c>
       <c r="B281" s="50" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="C281" s="62" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D281" s="46" t="s">
         <v>5</v>
@@ -11090,10 +10984,10 @@
         <v>279</v>
       </c>
       <c r="B282" s="50" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="C282" s="62" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D282" s="46" t="s">
         <v>5</v>
@@ -11116,10 +11010,10 @@
         <v>280</v>
       </c>
       <c r="B283" s="50" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="C283" s="62" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D283" s="46" t="s">
         <v>5</v>
@@ -11142,10 +11036,10 @@
         <v>281</v>
       </c>
       <c r="B284" s="50" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="C284" s="62" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D284" s="46" t="s">
         <v>5</v>
@@ -11168,10 +11062,10 @@
         <v>282</v>
       </c>
       <c r="B285" s="50" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="C285" s="62" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D285" s="46" t="s">
         <v>5</v>
@@ -11194,10 +11088,10 @@
         <v>283</v>
       </c>
       <c r="B286" s="50" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="C286" s="62" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D286" s="46" t="s">
         <v>5</v>
@@ -11220,10 +11114,10 @@
         <v>284</v>
       </c>
       <c r="B287" s="50" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="C287" s="62" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D287" s="46" t="s">
         <v>5</v>
@@ -11246,10 +11140,10 @@
         <v>285</v>
       </c>
       <c r="B288" s="50" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="C288" s="62" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D288" s="46" t="s">
         <v>5</v>
@@ -11272,10 +11166,10 @@
         <v>286</v>
       </c>
       <c r="B289" s="50" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="C289" s="62" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D289" s="46" t="s">
         <v>5</v>
@@ -11298,10 +11192,10 @@
         <v>287</v>
       </c>
       <c r="B290" s="50" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="C290" s="62" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D290" s="46" t="s">
         <v>5</v>

</xml_diff>